<commit_message>
fix(tabs): template says narrative_file replaces the summary Comments rows
The Comments sheet now says a narrative_file Word document replaces
_BACKGROUND and _EXECUTIVE_SUMMARY, and what formatting those two rows
support (each line a paragraph, "- " or "* " a bullet). The shipped template
is regenerated: only those three cells changed, 20 dropdowns, no drawing
parts. A new test fails whenever the shipped template differs from a fresh
generation, which is how it fell ten Settings rows behind before.

The stage 3 handover records the independent review fixes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/tabs/templates/Crosstab_Config_Template.xlsx
+++ b/modules/tabs/templates/Crosstab_Config_Template.xlsx
@@ -1379,7 +1379,7 @@
     <t xml:space="preserve">Question Comments &amp; Report Text</t>
   </si>
   <si>
-    <t xml:space="preserve">Add question-specific comments and report narrative sections. Use _BACKGROUND, _EXECUTIVE_SUMMARY and _REPORT_CONSTRUCTION for report sections.</t>
+    <t xml:space="preserve">Add question-specific comments and report narrative sections. Use _BACKGROUND, _EXECUTIVE_SUMMARY and _REPORT_CONSTRUCTION for report sections. A Word document named in the Settings sheet's narrative_file replaces _BACKGROUND and _EXECUTIVE_SUMMARY.</t>
   </si>
   <si>
     <t xml:space="preserve">Comment</t>
@@ -1391,10 +1391,10 @@
     <t xml:space="preserve">Headline</t>
   </si>
   <si>
-    <t xml:space="preserve">[REQUIRED] Question code to attach comment to, or _BACKGROUND / _EXECUTIVE_SUMMARY / _REPORT_CONSTRUCTION for report sections. A QUAL_ code targets the Qualitative tab instead of the crosstab card: QUAL_ plus the coded-comment worksheet name, uppercased, non-alphanumerics as underscores (sheet 'Q02Comment' -&gt; QUAL_Q02COMMENT). The Qualitative page prints the exact code in its empty insight box. Banner is ignored on a QUAL_ row.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[REQUIRED] Comment text. Supports markdown for HTML reports (bold, bullets, links).</t>
+    <t xml:space="preserve">[REQUIRED] Question code to attach comment to, or _BACKGROUND / _EXECUTIVE_SUMMARY / _REPORT_CONSTRUCTION for report sections (_BACKGROUND and _EXECUTIVE_SUMMARY are used only when the Settings sheet's narrative_file is blank). A QUAL_ code targets the Qualitative tab instead of the crosstab card: QUAL_ plus the coded-comment worksheet name, uppercased, non-alphanumerics as underscores (sheet 'Q02Comment' -&gt; QUAL_Q02COMMENT). The Qualitative page prints the exact code in its empty insight box. Banner is ignored on a QUAL_ row.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[REQUIRED] Comment text. Supports markdown for HTML reports (bold, bullets, links). In _BACKGROUND and _EXECUTIVE_SUMMARY each line is its own paragraph and a line starting "- " or "* " is a bullet; nothing else is formatted.</t>
   </si>
   <si>
     <t xml:space="preserve">[Optional] Optional: specific banner column this comment applies to. Leave blank for all banners.</t>

</xml_diff>